<commit_message>
commit the updated script for the pawning
</commit_message>
<xml_diff>
--- a/src/test/resources/TEST_DATA/PawningData.xlsx
+++ b/src/test/resources/TEST_DATA/PawningData.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>maxiumAmount</t>
   </si>
@@ -42,6 +42,12 @@
     <t>correctAmount</t>
   </si>
   <si>
+    <t>successMsg</t>
+  </si>
+  <si>
+    <t>maxRetries</t>
+  </si>
+  <si>
     <t>100000</t>
   </si>
   <si>
@@ -57,10 +63,16 @@
     <t>4000</t>
   </si>
   <si>
-    <t xml:space="preserve">Insufficient balance. Maximum available: LKR 2926.48</t>
+    <t xml:space="preserve">Insufficient balance. Maximum available:</t>
   </si>
   <si>
     <t xml:space="preserve">1022 5214 6593</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Payment success</t>
+  </si>
+  <si>
+    <t>3</t>
   </si>
 </sst>
 </file>
@@ -95,10 +107,8 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
@@ -614,26 +624,28 @@
     <col min="5" max="5" style="1" width="9.140625"/>
     <col customWidth="1" min="6" max="6" style="1" width="54.140625"/>
     <col customWidth="1" min="7" max="7" style="1" width="28.140625"/>
-    <col min="8" max="16384" style="1" width="9.140625"/>
+    <col customWidth="1" min="8" max="8" style="1" width="17.140625"/>
+    <col customWidth="1" min="9" max="9" style="1" width="19.7109375"/>
+    <col min="10" max="16384" style="1" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
@@ -641,32 +653,44 @@
       </c>
       <c r="H1" s="1" t="s">
         <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>15</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H2" s="1">
         <v>100</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>